<commit_message>
Export the name of outliers in the bar graph table to an Excel file. The order of the outliers in the table is based on their rank in the bar graph.
</commit_message>
<xml_diff>
--- a/results/bar_graph_table.xlsx
+++ b/results/bar_graph_table.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ardal\Desktop\notebooks for GitHub\ai-compound-target-extractor\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61507C27-1DD2-4C8D-9F41-AF6F184AB3D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4F7AFA8-1000-4E3C-8D51-78429E1C0F0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-107" yWindow="-107" windowWidth="20847" windowHeight="12401" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AA$20</definedName>
+  </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
@@ -589,12 +592,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -624,11 +633,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1082,7 +1092,7 @@
       <c r="K2" t="s">
         <v>76</v>
       </c>
-      <c r="L2" t="s">
+      <c r="L2" s="2" t="s">
         <v>87</v>
       </c>
       <c r="M2" t="s">
@@ -1094,7 +1104,7 @@
       <c r="O2" t="s">
         <v>108</v>
       </c>
-      <c r="P2" t="s">
+      <c r="P2" s="2" t="s">
         <v>111</v>
       </c>
       <c r="Q2" t="s">
@@ -1115,7 +1125,7 @@
       <c r="V2" t="s">
         <v>146</v>
       </c>
-      <c r="W2" t="s">
+      <c r="W2" s="2" t="s">
         <v>150</v>
       </c>
       <c r="X2" t="s">
@@ -1177,7 +1187,7 @@
       <c r="R3" t="s">
         <v>121</v>
       </c>
-      <c r="S3" t="s">
+      <c r="S3" s="2" t="s">
         <v>122</v>
       </c>
       <c r="U3" t="s">
@@ -1233,7 +1243,7 @@
       <c r="N4" t="s">
         <v>99</v>
       </c>
-      <c r="O4" t="s">
+      <c r="O4" s="2" t="s">
         <v>110</v>
       </c>
       <c r="P4" t="s">
@@ -1280,7 +1290,7 @@
       <c r="I5" t="s">
         <v>68</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="2" t="s">
         <v>73</v>
       </c>
       <c r="K5" t="s">
@@ -1488,7 +1498,7 @@
       <c r="N10" t="s">
         <v>105</v>
       </c>
-      <c r="P10" t="s">
+      <c r="P10" s="2" t="s">
         <v>113</v>
       </c>
       <c r="S10" t="s">
@@ -1520,13 +1530,13 @@
       <c r="S11" t="s">
         <v>127</v>
       </c>
-      <c r="U11" t="s">
+      <c r="U11" s="2" t="s">
         <v>144</v>
       </c>
       <c r="X11" t="s">
         <v>164</v>
       </c>
-      <c r="AA11" t="s">
+      <c r="AA11" s="2" t="s">
         <v>110</v>
       </c>
     </row>
@@ -1546,13 +1556,13 @@
       <c r="S12" t="s">
         <v>128</v>
       </c>
-      <c r="U12" t="s">
+      <c r="U12" s="2" t="s">
         <v>145</v>
       </c>
       <c r="X12" t="s">
         <v>165</v>
       </c>
-      <c r="AA12" t="s">
+      <c r="AA12" s="2" t="s">
         <v>181</v>
       </c>
     </row>
@@ -1593,7 +1603,7 @@
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="A16" s="2" t="s">
         <v>41</v>
       </c>
       <c r="S16" t="s">
@@ -1606,12 +1616,12 @@
       </c>
     </row>
     <row r="18" spans="19:19" x14ac:dyDescent="0.3">
-      <c r="S18" t="s">
+      <c r="S18" s="2" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="19" spans="19:19" x14ac:dyDescent="0.3">
-      <c r="S19" t="s">
+      <c r="S19" s="2" t="s">
         <v>134</v>
       </c>
     </row>
@@ -1621,6 +1631,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AA20" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>